<commit_message>
Se añadio la base de datos completa, a nivel municipio, zona metropolitana, regional, estatal y referencias
</commit_message>
<xml_diff>
--- a/Output/Infografia_Base_Regional_2026_Enero.xlsx
+++ b/Output/Infografia_Base_Regional_2026_Enero.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="777">
   <si>
     <t xml:space="preserve">CVE_MUN</t>
   </si>
@@ -2105,6 +2105,42 @@
     <t xml:space="preserve">Popoluca insuficientemente especificado</t>
   </si>
   <si>
+    <t xml:space="preserve">Lenguas Indigenas Top 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lenguas Indigenas Top 5 Conteo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada conteo 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada conteo 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada conteo 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada conteo 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lengua Indigena más hablada conteo 5</t>
+  </si>
+  <si>
     <t xml:space="preserve">13003, 13009, 13023, 13041, 13050, 13054, 13055</t>
   </si>
   <si>
@@ -2126,6 +2162,9 @@
     <t xml:space="preserve">Medio</t>
   </si>
   <si>
+    <t xml:space="preserve">Otomí, Náhuatl, Mixteco, Totonaco, Zapoteco</t>
+  </si>
+  <si>
     <t xml:space="preserve">13007, 13008, 13021, 13061, 13072</t>
   </si>
   <si>
@@ -2141,6 +2180,9 @@
     <t xml:space="preserve">Bajo</t>
   </si>
   <si>
+    <t xml:space="preserve">Náhuatl, Otomí, Zapoteco, Totonaco, Mazahua</t>
+  </si>
+  <si>
     <t xml:space="preserve">13011, 13014, 13025, 13026, 13028, 13032, 13034, 13046, 13073, 13078, 13080</t>
   </si>
   <si>
@@ -2159,6 +2201,9 @@
     <t xml:space="preserve">Alto</t>
   </si>
   <si>
+    <t xml:space="preserve">Náhuatl, No especificado lengua indigena, Huasteco, Otomí, Totonaco</t>
+  </si>
+  <si>
     <t xml:space="preserve">13017, 13029, 13044, 13059</t>
   </si>
   <si>
@@ -2174,6 +2219,9 @@
     <t xml:space="preserve">2do año de Secundaria</t>
   </si>
   <si>
+    <t xml:space="preserve">Otomí, Náhuatl, Mixteco, No especificado lengua indigena, Zapoteco</t>
+  </si>
+  <si>
     <t xml:space="preserve">13006, 13015, 13019, 13030, 13043, 13058, 13084</t>
   </si>
   <si>
@@ -2186,6 +2234,9 @@
     <t xml:space="preserve">Santuario de Mapethé, Boxiza, Asthar</t>
   </si>
   <si>
+    <t xml:space="preserve">Otomí, Náhuatl, No especificado lengua indigena, Mixteco, Mazahua</t>
+  </si>
+  <si>
     <t xml:space="preserve">13018, 13031, 13040, 13047, 13049</t>
   </si>
   <si>
@@ -2204,6 +2255,9 @@
     <t xml:space="preserve">Muy alto</t>
   </si>
   <si>
+    <t xml:space="preserve">Náhuatl, Otomí, Huasteco, Mixteco, Zapoteco</t>
+  </si>
+  <si>
     <t xml:space="preserve">13022, 13024, 13038, 13039, 13045, 13051</t>
   </si>
   <si>
@@ -2216,6 +2270,9 @@
     <t xml:space="preserve">Parque Estatal Bosque El Hiloche</t>
   </si>
   <si>
+    <t xml:space="preserve">Náhuatl, Otomí, Totonaco, Zapoteco, Mixteco</t>
+  </si>
+  <si>
     <t xml:space="preserve">13048, 13052, 13082</t>
   </si>
   <si>
@@ -2255,6 +2312,9 @@
     <t xml:space="preserve">El Xhinfi y La Sierrita, Ejido Ajacuba, El Zoológico, Vega de Madero, Cerro Lobo, El Sabino, El Tigre y El Laurel, Cerro Grande</t>
   </si>
   <si>
+    <t xml:space="preserve">Otomí, Náhuatl, Zapoteco, Mixteco, Totonaco</t>
+  </si>
+  <si>
     <t xml:space="preserve">13001, 13002, 13004, 13016, 13027, 13035, 13053, 13056, 13057, 13060, 13077</t>
   </si>
   <si>
@@ -2267,6 +2327,9 @@
     <t xml:space="preserve">Mixquiapan, El Campanario, San Ignacio-El Coyuco, La Piedra, Chicamole, Medio Monte, Cerro La Paila-El Susto, Cerro La Paila-Matías Rodríguez, La Lagunilla</t>
   </si>
   <si>
+    <t xml:space="preserve">Otomí, Náhuatl, Tepehua, Totonaco, Mixteco</t>
+  </si>
+  <si>
     <t xml:space="preserve">13012, 13020, 13033, 13036, 13037, 13042, 13062, 13068, 13071, 13079, 13081</t>
   </si>
   <si>
@@ -2277,6 +2340,9 @@
   </si>
   <si>
     <t xml:space="preserve">Arroyo Nogales, Cruz de Plata, Plan Grande</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Náhuatl, Otomí, Zapoteco, Huasteco, Totonaco</t>
   </si>
 </sst>
 </file>
@@ -4697,16 +4763,52 @@
       <c r="ZU1" t="s">
         <v>696</v>
       </c>
+      <c r="ZV1" t="s">
+        <v>697</v>
+      </c>
+      <c r="ZW1" t="s">
+        <v>698</v>
+      </c>
+      <c r="ZX1" t="s">
+        <v>699</v>
+      </c>
+      <c r="ZY1" t="s">
+        <v>700</v>
+      </c>
+      <c r="ZZ1" t="s">
+        <v>701</v>
+      </c>
+      <c r="AAA1" t="s">
+        <v>702</v>
+      </c>
+      <c r="AAB1" t="s">
+        <v>703</v>
+      </c>
+      <c r="AAC1" t="s">
+        <v>704</v>
+      </c>
+      <c r="AAD1" t="s">
+        <v>705</v>
+      </c>
+      <c r="AAE1" t="s">
+        <v>706</v>
+      </c>
+      <c r="AAF1" t="s">
+        <v>707</v>
+      </c>
+      <c r="AAG1" t="s">
+        <v>708</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>697</v>
+        <v>709</v>
       </c>
       <c r="B2" t="s">
-        <v>698</v>
+        <v>710</v>
       </c>
       <c r="C2" t="s">
-        <v>699</v>
+        <v>711</v>
       </c>
       <c r="D2" t="n">
         <v>1196.21807022</v>
@@ -5249,7 +5351,7 @@
         <v>2</v>
       </c>
       <c r="GB2" t="s">
-        <v>700</v>
+        <v>712</v>
       </c>
       <c r="GC2" t="n">
         <v>150912</v>
@@ -5441,7 +5543,7 @@
         <v>9.66142857142857</v>
       </c>
       <c r="IN2" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
       <c r="IO2" t="n">
         <v>182363</v>
@@ -5582,13 +5684,13 @@
         <v>57.0143290373989</v>
       </c>
       <c r="KI2" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="KJ2" t="n">
         <v>62.6278128571429</v>
       </c>
       <c r="KK2" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="KL2" t="n">
         <v>47</v>
@@ -6789,17 +6891,53 @@
       </c>
       <c r="ZU2" t="n">
         <v>1</v>
+      </c>
+      <c r="ZV2" t="s">
+        <v>716</v>
+      </c>
+      <c r="ZW2" t="n">
+        <v>38818</v>
+      </c>
+      <c r="ZX2" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZY2" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZZ2" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAA2" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAB2" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAC2" t="n">
+        <v>37321</v>
+      </c>
+      <c r="AAD2" t="n">
+        <v>1137</v>
+      </c>
+      <c r="AAE2" t="n">
+        <v>161</v>
+      </c>
+      <c r="AAF2" t="n">
+        <v>104</v>
+      </c>
+      <c r="AAG2" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>704</v>
+        <v>717</v>
       </c>
       <c r="B3" t="s">
-        <v>705</v>
+        <v>718</v>
       </c>
       <c r="C3" t="s">
-        <v>706</v>
+        <v>719</v>
       </c>
       <c r="D3" t="n">
         <v>1043.39108633</v>
@@ -7342,7 +7480,7 @@
         <v>9</v>
       </c>
       <c r="GB3" t="s">
-        <v>707</v>
+        <v>720</v>
       </c>
       <c r="GC3" t="n">
         <v>120400</v>
@@ -7534,7 +7672,7 @@
         <v>9.58</v>
       </c>
       <c r="IN3" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
       <c r="IO3" t="n">
         <v>108221</v>
@@ -7675,13 +7813,13 @@
         <v>58.0188368597015</v>
       </c>
       <c r="KI3" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="KJ3" t="n">
         <v>64.016792</v>
       </c>
       <c r="KK3" t="s">
-        <v>708</v>
+        <v>721</v>
       </c>
       <c r="KL3" t="n">
         <v>40</v>
@@ -8882,17 +9020,53 @@
       </c>
       <c r="ZU3" t="n">
         <v>0</v>
+      </c>
+      <c r="ZV3" t="s">
+        <v>722</v>
+      </c>
+      <c r="ZW3" t="n">
+        <v>1169</v>
+      </c>
+      <c r="ZX3" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZY3" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZZ3" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAA3" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAB3" t="s">
+        <v>659</v>
+      </c>
+      <c r="AAC3" t="n">
+        <v>788</v>
+      </c>
+      <c r="AAD3" t="n">
+        <v>244</v>
+      </c>
+      <c r="AAE3" t="n">
+        <v>60</v>
+      </c>
+      <c r="AAF3" t="n">
+        <v>45</v>
+      </c>
+      <c r="AAG3" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>709</v>
+        <v>723</v>
       </c>
       <c r="B4" t="s">
-        <v>710</v>
+        <v>724</v>
       </c>
       <c r="C4" t="s">
-        <v>711</v>
+        <v>725</v>
       </c>
       <c r="D4" t="n">
         <v>2368.92972556</v>
@@ -9435,7 +9609,7 @@
         <v>6</v>
       </c>
       <c r="GB4" t="s">
-        <v>712</v>
+        <v>726</v>
       </c>
       <c r="GC4" t="n">
         <v>181100</v>
@@ -9627,7 +9801,7 @@
         <v>7.24727272727273</v>
       </c>
       <c r="IN4" t="s">
-        <v>713</v>
+        <v>727</v>
       </c>
       <c r="IO4" t="n">
         <v>237487</v>
@@ -9768,13 +9942,13 @@
         <v>51.9375548924334</v>
       </c>
       <c r="KI4" t="s">
-        <v>714</v>
+        <v>728</v>
       </c>
       <c r="KJ4" t="n">
         <v>64.5369590909091</v>
       </c>
       <c r="KK4" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="KL4" t="n">
         <v>69</v>
@@ -10975,17 +11149,53 @@
       </c>
       <c r="ZU4" t="n">
         <v>6</v>
+      </c>
+      <c r="ZV4" t="s">
+        <v>729</v>
+      </c>
+      <c r="ZW4" t="n">
+        <v>254269</v>
+      </c>
+      <c r="ZX4" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZY4" t="s">
+        <v>693</v>
+      </c>
+      <c r="ZZ4" t="s">
+        <v>674</v>
+      </c>
+      <c r="AAA4" t="s">
+        <v>658</v>
+      </c>
+      <c r="AAB4" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAC4" t="n">
+        <v>253015</v>
+      </c>
+      <c r="AAD4" t="n">
+        <v>620</v>
+      </c>
+      <c r="AAE4" t="n">
+        <v>342</v>
+      </c>
+      <c r="AAF4" t="n">
+        <v>190</v>
+      </c>
+      <c r="AAG4" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>715</v>
+        <v>730</v>
       </c>
       <c r="B5" t="s">
-        <v>716</v>
+        <v>731</v>
       </c>
       <c r="C5" t="s">
-        <v>717</v>
+        <v>732</v>
       </c>
       <c r="D5" t="n">
         <v>1805.41999614</v>
@@ -11528,7 +11738,7 @@
         <v>6</v>
       </c>
       <c r="GB5" t="s">
-        <v>718</v>
+        <v>733</v>
       </c>
       <c r="GC5" t="n">
         <v>52900</v>
@@ -11720,7 +11930,7 @@
         <v>8.1225</v>
       </c>
       <c r="IN5" t="s">
-        <v>719</v>
+        <v>734</v>
       </c>
       <c r="IO5" t="n">
         <v>85638</v>
@@ -11861,13 +12071,13 @@
         <v>54.5435061244546</v>
       </c>
       <c r="KI5" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="KJ5" t="n">
         <v>61.357195</v>
       </c>
       <c r="KK5" t="s">
-        <v>714</v>
+        <v>728</v>
       </c>
       <c r="KL5" t="n">
         <v>94</v>
@@ -13068,17 +13278,53 @@
       </c>
       <c r="ZU5" t="n">
         <v>0</v>
+      </c>
+      <c r="ZV5" t="s">
+        <v>735</v>
+      </c>
+      <c r="ZW5" t="n">
+        <v>8545</v>
+      </c>
+      <c r="ZX5" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZY5" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZZ5" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAA5" t="s">
+        <v>693</v>
+      </c>
+      <c r="AAB5" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAC5" t="n">
+        <v>8120</v>
+      </c>
+      <c r="AAD5" t="n">
+        <v>277</v>
+      </c>
+      <c r="AAE5" t="n">
+        <v>58</v>
+      </c>
+      <c r="AAF5" t="n">
+        <v>53</v>
+      </c>
+      <c r="AAG5" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>720</v>
+        <v>736</v>
       </c>
       <c r="B6" t="s">
-        <v>721</v>
+        <v>737</v>
       </c>
       <c r="C6" t="s">
-        <v>722</v>
+        <v>738</v>
       </c>
       <c r="D6" t="n">
         <v>3098.78729034</v>
@@ -13621,7 +13867,7 @@
         <v>3</v>
       </c>
       <c r="GB6" t="s">
-        <v>723</v>
+        <v>739</v>
       </c>
       <c r="GC6" t="n">
         <v>149060</v>
@@ -13813,7 +14059,7 @@
         <v>8.58142857142857</v>
       </c>
       <c r="IN6" t="s">
-        <v>719</v>
+        <v>734</v>
       </c>
       <c r="IO6" t="n">
         <v>161435</v>
@@ -13954,13 +14200,13 @@
         <v>54.9605453921261</v>
       </c>
       <c r="KI6" t="s">
-        <v>708</v>
+        <v>721</v>
       </c>
       <c r="KJ6" t="n">
         <v>60.1650757142857</v>
       </c>
       <c r="KK6" t="s">
-        <v>714</v>
+        <v>728</v>
       </c>
       <c r="KL6" t="n">
         <v>123</v>
@@ -15161,17 +15407,53 @@
       </c>
       <c r="ZU6" t="n">
         <v>3</v>
+      </c>
+      <c r="ZV6" t="s">
+        <v>740</v>
+      </c>
+      <c r="ZW6" t="n">
+        <v>119509</v>
+      </c>
+      <c r="ZX6" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZY6" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZZ6" t="s">
+        <v>693</v>
+      </c>
+      <c r="AAA6" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAB6" t="s">
+        <v>659</v>
+      </c>
+      <c r="AAC6" t="n">
+        <v>117239</v>
+      </c>
+      <c r="AAD6" t="n">
+        <v>1624</v>
+      </c>
+      <c r="AAE6" t="n">
+        <v>326</v>
+      </c>
+      <c r="AAF6" t="n">
+        <v>182</v>
+      </c>
+      <c r="AAG6" t="n">
+        <v>138</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>724</v>
+        <v>741</v>
       </c>
       <c r="B7" t="s">
-        <v>725</v>
+        <v>742</v>
       </c>
       <c r="C7" t="s">
-        <v>726</v>
+        <v>743</v>
       </c>
       <c r="D7" t="n">
         <v>1478.88017612</v>
@@ -15714,7 +15996,7 @@
         <v>1</v>
       </c>
       <c r="GB7" t="s">
-        <v>727</v>
+        <v>744</v>
       </c>
       <c r="GC7" t="n">
         <v>35500</v>
@@ -15906,7 +16188,7 @@
         <v>6.96</v>
       </c>
       <c r="IN7" t="s">
-        <v>728</v>
+        <v>745</v>
       </c>
       <c r="IO7" t="n">
         <v>48138</v>
@@ -16047,13 +16329,13 @@
         <v>51.9959349236018</v>
       </c>
       <c r="KI7" t="s">
-        <v>714</v>
+        <v>728</v>
       </c>
       <c r="KJ7" t="n">
         <v>55.53546</v>
       </c>
       <c r="KK7" t="s">
-        <v>729</v>
+        <v>746</v>
       </c>
       <c r="KL7" t="n">
         <v>16</v>
@@ -17254,17 +17536,53 @@
       </c>
       <c r="ZU7" t="n">
         <v>0</v>
+      </c>
+      <c r="ZV7" t="s">
+        <v>747</v>
+      </c>
+      <c r="ZW7" t="n">
+        <v>3870</v>
+      </c>
+      <c r="ZX7" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZY7" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZZ7" t="s">
+        <v>674</v>
+      </c>
+      <c r="AAA7" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAB7" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAC7" t="n">
+        <v>3249</v>
+      </c>
+      <c r="AAD7" t="n">
+        <v>490</v>
+      </c>
+      <c r="AAE7" t="n">
+        <v>75</v>
+      </c>
+      <c r="AAF7" t="n">
+        <v>35</v>
+      </c>
+      <c r="AAG7" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>730</v>
+        <v>748</v>
       </c>
       <c r="B8" t="s">
-        <v>731</v>
+        <v>749</v>
       </c>
       <c r="C8" t="s">
-        <v>732</v>
+        <v>750</v>
       </c>
       <c r="D8" t="n">
         <v>883.0237455</v>
@@ -17807,7 +18125,7 @@
         <v>1</v>
       </c>
       <c r="GB8" t="s">
-        <v>733</v>
+        <v>751</v>
       </c>
       <c r="GC8" t="n">
         <v>127250</v>
@@ -17999,7 +18317,7 @@
         <v>9.18666666666667</v>
       </c>
       <c r="IN8" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
       <c r="IO8" t="n">
         <v>205289</v>
@@ -18140,13 +18458,13 @@
         <v>56.2358668625057</v>
       </c>
       <c r="KI8" t="s">
-        <v>708</v>
+        <v>721</v>
       </c>
       <c r="KJ8" t="n">
         <v>63.0539483333333</v>
       </c>
       <c r="KK8" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="KL8" t="n">
         <v>270</v>
@@ -19347,17 +19665,53 @@
       </c>
       <c r="ZU8" t="n">
         <v>9</v>
+      </c>
+      <c r="ZV8" t="s">
+        <v>752</v>
+      </c>
+      <c r="ZW8" t="n">
+        <v>11348</v>
+      </c>
+      <c r="ZX8" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZY8" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZZ8" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAA8" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAB8" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAC8" t="n">
+        <v>8268</v>
+      </c>
+      <c r="AAD8" t="n">
+        <v>2552</v>
+      </c>
+      <c r="AAE8" t="n">
+        <v>196</v>
+      </c>
+      <c r="AAF8" t="n">
+        <v>169</v>
+      </c>
+      <c r="AAG8" t="n">
+        <v>163</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>734</v>
+        <v>753</v>
       </c>
       <c r="B9" t="s">
-        <v>735</v>
+        <v>754</v>
       </c>
       <c r="C9" t="s">
-        <v>736</v>
+        <v>755</v>
       </c>
       <c r="D9" t="n">
         <v>556.65238685</v>
@@ -19900,7 +20254,7 @@
         <v>1</v>
       </c>
       <c r="GB9" t="s">
-        <v>737</v>
+        <v>756</v>
       </c>
       <c r="GC9" t="n">
         <v>234481</v>
@@ -20092,7 +20446,7 @@
         <v>10.05</v>
       </c>
       <c r="IN9" t="s">
-        <v>738</v>
+        <v>757</v>
       </c>
       <c r="IO9" t="n">
         <v>292744</v>
@@ -20233,13 +20587,13 @@
         <v>58.1789685758806</v>
       </c>
       <c r="KI9" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="KJ9" t="n">
         <v>64.12493</v>
       </c>
       <c r="KK9" t="s">
-        <v>708</v>
+        <v>721</v>
       </c>
       <c r="KL9" t="n">
         <v>52</v>
@@ -21440,17 +21794,53 @@
       </c>
       <c r="ZU9" t="n">
         <v>18</v>
+      </c>
+      <c r="ZV9" t="s">
+        <v>752</v>
+      </c>
+      <c r="ZW9" t="n">
+        <v>26175</v>
+      </c>
+      <c r="ZX9" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZY9" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZZ9" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAA9" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAB9" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAC9" t="n">
+        <v>19429</v>
+      </c>
+      <c r="AAD9" t="n">
+        <v>5730</v>
+      </c>
+      <c r="AAE9" t="n">
+        <v>405</v>
+      </c>
+      <c r="AAF9" t="n">
+        <v>334</v>
+      </c>
+      <c r="AAG9" t="n">
+        <v>277</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>739</v>
+        <v>758</v>
       </c>
       <c r="B10" t="s">
-        <v>740</v>
+        <v>759</v>
       </c>
       <c r="C10" t="s">
-        <v>741</v>
+        <v>760</v>
       </c>
       <c r="D10" t="n">
         <v>616.2235994</v>
@@ -21993,7 +22383,7 @@
         <v>2</v>
       </c>
       <c r="GB10" t="s">
-        <v>742</v>
+        <v>761</v>
       </c>
       <c r="GC10" t="n">
         <v>225000</v>
@@ -22185,7 +22575,7 @@
         <v>9.8975</v>
       </c>
       <c r="IN10" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
       <c r="IO10" t="n">
         <v>191559</v>
@@ -22326,13 +22716,13 @@
         <v>58.4093063825559</v>
       </c>
       <c r="KI10" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="KJ10" t="n">
         <v>64.66364</v>
       </c>
       <c r="KK10" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="KL10" t="n">
         <v>24</v>
@@ -23533,17 +23923,53 @@
       </c>
       <c r="ZU10" t="n">
         <v>41</v>
+      </c>
+      <c r="ZV10" t="s">
+        <v>752</v>
+      </c>
+      <c r="ZW10" t="n">
+        <v>7908</v>
+      </c>
+      <c r="ZX10" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZY10" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZZ10" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAA10" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAB10" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAC10" t="n">
+        <v>5211</v>
+      </c>
+      <c r="AAD10" t="n">
+        <v>1136</v>
+      </c>
+      <c r="AAE10" t="n">
+        <v>718</v>
+      </c>
+      <c r="AAF10" t="n">
+        <v>450</v>
+      </c>
+      <c r="AAG10" t="n">
+        <v>393</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>743</v>
+        <v>762</v>
       </c>
       <c r="B11" t="s">
-        <v>744</v>
+        <v>763</v>
       </c>
       <c r="C11" t="s">
-        <v>745</v>
+        <v>764</v>
       </c>
       <c r="D11" t="n">
         <v>1539.93269056</v>
@@ -24086,7 +24512,7 @@
         <v>8</v>
       </c>
       <c r="GB11" t="s">
-        <v>746</v>
+        <v>765</v>
       </c>
       <c r="GC11" t="n">
         <v>232286</v>
@@ -24278,7 +24704,7 @@
         <v>9.358</v>
       </c>
       <c r="IN11" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
       <c r="IO11" t="n">
         <v>332644</v>
@@ -24419,13 +24845,13 @@
         <v>57.8016158903057</v>
       </c>
       <c r="KI11" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="KJ11" t="n">
         <v>64.335787</v>
       </c>
       <c r="KK11" t="s">
-        <v>708</v>
+        <v>721</v>
       </c>
       <c r="KL11" t="n">
         <v>154</v>
@@ -25626,17 +26052,53 @@
       </c>
       <c r="ZU11" t="n">
         <v>22</v>
+      </c>
+      <c r="ZV11" t="s">
+        <v>766</v>
+      </c>
+      <c r="ZW11" t="n">
+        <v>10283</v>
+      </c>
+      <c r="ZX11" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZY11" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZZ11" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAA11" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAB11" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAC11" t="n">
+        <v>7024</v>
+      </c>
+      <c r="AAD11" t="n">
+        <v>1876</v>
+      </c>
+      <c r="AAE11" t="n">
+        <v>714</v>
+      </c>
+      <c r="AAF11" t="n">
+        <v>374</v>
+      </c>
+      <c r="AAG11" t="n">
+        <v>295</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>747</v>
+        <v>767</v>
       </c>
       <c r="B12" t="s">
-        <v>748</v>
+        <v>768</v>
       </c>
       <c r="C12" t="s">
-        <v>749</v>
+        <v>769</v>
       </c>
       <c r="D12" t="n">
         <v>2590.08688488</v>
@@ -26179,7 +26641,7 @@
         <v>9</v>
       </c>
       <c r="GB12" t="s">
-        <v>750</v>
+        <v>770</v>
       </c>
       <c r="GC12" t="n">
         <v>243036</v>
@@ -26371,7 +26833,7 @@
         <v>7.72818181818182</v>
       </c>
       <c r="IN12" t="s">
-        <v>713</v>
+        <v>727</v>
       </c>
       <c r="IO12" t="n">
         <v>314105</v>
@@ -26512,13 +26974,13 @@
         <v>53.5448008477015</v>
       </c>
       <c r="KI12" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="KJ12" t="n">
         <v>63.0708572727273</v>
       </c>
       <c r="KK12" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="KL12" t="n">
         <v>117</v>
@@ -27719,17 +28181,53 @@
       </c>
       <c r="ZU12" t="n">
         <v>15</v>
+      </c>
+      <c r="ZV12" t="s">
+        <v>771</v>
+      </c>
+      <c r="ZW12" t="n">
+        <v>67876</v>
+      </c>
+      <c r="ZX12" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZY12" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZZ12" t="s">
+        <v>687</v>
+      </c>
+      <c r="AAA12" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAB12" t="s">
+        <v>671</v>
+      </c>
+      <c r="AAC12" t="n">
+        <v>36846</v>
+      </c>
+      <c r="AAD12" t="n">
+        <v>27149</v>
+      </c>
+      <c r="AAE12" t="n">
+        <v>3291</v>
+      </c>
+      <c r="AAF12" t="n">
+        <v>469</v>
+      </c>
+      <c r="AAG12" t="n">
+        <v>121</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>751</v>
+        <v>772</v>
       </c>
       <c r="B13" t="s">
-        <v>752</v>
+        <v>773</v>
       </c>
       <c r="C13" t="s">
-        <v>753</v>
+        <v>774</v>
       </c>
       <c r="D13" t="n">
         <v>3643.89753021</v>
@@ -28272,7 +28770,7 @@
         <v>3</v>
       </c>
       <c r="GB13" t="s">
-        <v>754</v>
+        <v>775</v>
       </c>
       <c r="GC13" t="n">
         <v>63998</v>
@@ -28464,7 +28962,7 @@
         <v>7.58909090909091</v>
       </c>
       <c r="IN13" t="s">
-        <v>713</v>
+        <v>727</v>
       </c>
       <c r="IO13" t="n">
         <v>128594</v>
@@ -28605,13 +29103,13 @@
         <v>53.4693065141681</v>
       </c>
       <c r="KI13" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="KJ13" t="n">
         <v>62.1916354545455</v>
       </c>
       <c r="KK13" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="KL13" t="n">
         <v>51</v>
@@ -29812,6 +30310,42 @@
       </c>
       <c r="ZU13" t="n">
         <v>0</v>
+      </c>
+      <c r="ZV13" t="s">
+        <v>776</v>
+      </c>
+      <c r="ZW13" t="n">
+        <v>32581</v>
+      </c>
+      <c r="ZX13" t="s">
+        <v>656</v>
+      </c>
+      <c r="ZY13" t="s">
+        <v>658</v>
+      </c>
+      <c r="ZZ13" t="s">
+        <v>668</v>
+      </c>
+      <c r="AAA13" t="s">
+        <v>674</v>
+      </c>
+      <c r="AAB13" t="s">
+        <v>686</v>
+      </c>
+      <c r="AAC13" t="n">
+        <v>28986</v>
+      </c>
+      <c r="AAD13" t="n">
+        <v>3416</v>
+      </c>
+      <c r="AAE13" t="n">
+        <v>68</v>
+      </c>
+      <c r="AAF13" t="n">
+        <v>67</v>
+      </c>
+      <c r="AAG13" t="n">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>